<commit_message>
aggiunta file classifica challenge
</commit_message>
<xml_diff>
--- a/no-bounce-challenge.xlsx
+++ b/no-bounce-challenge.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Documents\GitHub\12orebosaro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA75BB6-D595-4D02-BE9E-CF84BEC98768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61FF13B4-2900-4486-9EC7-9E6A2F2AF320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Nome</t>
   </si>
@@ -34,12 +34,6 @@
   </si>
   <si>
     <t>Gol validi</t>
-  </si>
-  <si>
-    <t>Daniel</t>
-  </si>
-  <si>
-    <t>Marchi</t>
   </si>
 </sst>
 </file>
@@ -366,7 +360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -380,17 +374,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2">
-        <v>10</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>